<commit_message>
远征01 房型美术源入库（bridge_room v001/v002＋office_room v001＋db_room v001＋std_25x25 v001 共 457 件：.blend 源＋GLB＋PackedScene＋组件包＋构建清单，bridge_room v002 84.4MB/office_room 58.3MB/db_room 32.4MB 为已知最大入库件）＋整波清空与2秒间歇修复（Dungeon3D 独占波次队列与暂停感知 timer、波次 token 抵御过期/重复超时、离场幂等计数先于击杀事件、召唤预约可序列化重放、命运增援每房仅一次、HUD 独立波次栏；新增 verify_dungeon_wave_intermission 回归并注册 core）＋落点代理失败锁定（DungeonRoom3D 批量落点预检、非有限点返回内部失败码、本房失败锁随快照保存、probe_expedition_spawn_safety）＋墙面探针组 8 件（corner_relief／shared_wall_sides／wall_collision_audit／wall_facing_shots／wall_prefab_gallery／wall_relief／wall_tint_shots／wall_visual_facing）＋账本同步（场景账本 v001.xlsx、ledger_split_baseline.json、feature_registry）＋文档（远征关卡01设计、05.2 关卡版图、06 怪物与Boss、14 命运塔罗、MODULE_INDEX、CHANGELOG、新增开发日志 2026-09-26_room_wave_intermission）＋skill 双副本同步（新增 godot-export-pack-audit，更新 01-battle-room-type-art-authoring／godot-runtime-probe／shellstorm2-asset-ledger-row-authoring）
</commit_message>
<xml_diff>
--- a/assets/registry/ledgers/ShellStorm2_场景账本_v001.xlsx
+++ b/assets/registry/ledgers/ShellStorm2_场景账本_v001.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="总览" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="账本说明" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="资产主表" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="3D-场景通用" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="3D-设施" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="3D-其他" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="域变更日志" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="总览" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="账本说明" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="资产主表" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3D-场景通用" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3D-设施" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3D-其他" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="域变更日志" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'资产主表'!$A$5:$X$240</definedName>
@@ -1476,22 +1476,22 @@
     </row>
     <row r="6" ht="42" customHeight="1" s="60">
       <c r="A6" s="65">
-        <f>COUNTA('资产主表'!$A$6:$A$242)</f>
+        <f>COUNTA('资产主表'!$A$6:$A$246)</f>
         <v/>
       </c>
       <c r="B6" s="63" t="n"/>
       <c r="C6" s="65">
-        <f>COUNTIF('资产主表'!$K$6:$K$242,"已完成")+COUNTIF('资产主表'!$K$6:$K$242,"原型已接入")+COUNTIF('资产主表'!$K$6:$K$242,"正式美术已接入")+COUNTIF('资产主表'!$K$6:$K$242,"已优化并正式接入")+COUNTIF('资产主表'!$K$6:$K$242,"Blender源已完成")+COUNTIF('资产主表'!$K$6:$K$242,"已导入；优化完成")+COUNTIF('资产主表'!$K$6:$K$242,"白模源已完成；QA PASS")</f>
+        <f>COUNTIF('资产主表'!$K$6:$K$246,"已完成")+COUNTIF('资产主表'!$K$6:$K$246,"原型已接入")+COUNTIF('资产主表'!$K$6:$K$246,"正式美术已接入")+COUNTIF('资产主表'!$K$6:$K$246,"已优化并正式接入")+COUNTIF('资产主表'!$K$6:$K$246,"Blender源已完成")+COUNTIF('资产主表'!$K$6:$K$246,"已导入；优化完成")+COUNTIF('资产主表'!$K$6:$K$246,"白模源已完成；QA PASS")</f>
         <v/>
       </c>
       <c r="D6" s="63" t="n"/>
       <c r="E6" s="65">
-        <f>COUNTIF('资产主表'!$K$6:$K$242,"待制作")+COUNTIF('资产主表'!$K$6:$K$242,"程序占位")</f>
+        <f>COUNTIF('资产主表'!$K$6:$K$246,"待制作")+COUNTIF('资产主表'!$K$6:$K$246,"程序占位")</f>
         <v/>
       </c>
       <c r="F6" s="63" t="n"/>
       <c r="G6" s="65">
-        <f>COUNTIF('资产主表'!$S$6:$S$242,"重复")</f>
+        <f>COUNTIF('资产主表'!$S$6:$S$246,"重复")</f>
         <v/>
       </c>
       <c r="H6" s="63" t="n"/>
@@ -1560,11 +1560,11 @@
         </is>
       </c>
       <c r="B10" s="70">
-        <f>COUNTIF('资产主表'!$C$6:$C$242,A10)</f>
+        <f>COUNTIF('资产主表'!$C$6:$C$246,A10)</f>
         <v/>
       </c>
       <c r="C10" s="70">
-        <f>SUMPRODUCT(('资产主表'!$C$6:$C$242=A10)*(('资产主表'!$K$6:$K$242="已完成")+('资产主表'!$K$6:$K$242="原型已接入")+('资产主表'!$K$6:$K$242="正式美术已接入")+('资产主表'!$K$6:$K$242="已优化并正式接入")+('资产主表'!$K$6:$K$242="Blender源已完成")+('资产主表'!$K$6:$K$242="已导入；优化完成")+('资产主表'!$K$6:$K$242="白模源已完成；QA PASS")))</f>
+        <f>SUMPRODUCT(('资产主表'!$C$6:$C$246=A10)*(('资产主表'!$K$6:$K$246="已完成")+('资产主表'!$K$6:$K$246="原型已接入")+('资产主表'!$K$6:$K$246="正式美术已接入")+('资产主表'!$K$6:$K$246="已优化并正式接入")+('资产主表'!$K$6:$K$246="Blender源已完成")+('资产主表'!$K$6:$K$246="已导入；优化完成")+('资产主表'!$K$6:$K$246="白模源已完成；QA PASS")))</f>
         <v/>
       </c>
       <c r="D10" s="70" t="n"/>
@@ -1582,11 +1582,11 @@
         </is>
       </c>
       <c r="B11" s="70">
-        <f>COUNTIF('资产主表'!$C$6:$C$242,A11)</f>
+        <f>COUNTIF('资产主表'!$C$6:$C$246,A11)</f>
         <v/>
       </c>
       <c r="C11" s="70">
-        <f>SUMPRODUCT(('资产主表'!$C$6:$C$242=A11)*(('资产主表'!$K$6:$K$242="已完成")+('资产主表'!$K$6:$K$242="原型已接入")+('资产主表'!$K$6:$K$242="正式美术已接入")+('资产主表'!$K$6:$K$242="已优化并正式接入")+('资产主表'!$K$6:$K$242="Blender源已完成")+('资产主表'!$K$6:$K$242="已导入；优化完成")+('资产主表'!$K$6:$K$242="白模源已完成；QA PASS")))</f>
+        <f>SUMPRODUCT(('资产主表'!$C$6:$C$246=A11)*(('资产主表'!$K$6:$K$246="已完成")+('资产主表'!$K$6:$K$246="原型已接入")+('资产主表'!$K$6:$K$246="正式美术已接入")+('资产主表'!$K$6:$K$246="已优化并正式接入")+('资产主表'!$K$6:$K$246="Blender源已完成")+('资产主表'!$K$6:$K$246="已导入；优化完成")+('资产主表'!$K$6:$K$246="白模源已完成；QA PASS")))</f>
         <v/>
       </c>
       <c r="D11" s="70" t="n"/>
@@ -1604,11 +1604,11 @@
         </is>
       </c>
       <c r="B12" s="70">
-        <f>COUNTIF('资产主表'!$C$6:$C$242,A12)</f>
+        <f>COUNTIF('资产主表'!$C$6:$C$246,A12)</f>
         <v/>
       </c>
       <c r="C12" s="70">
-        <f>SUMPRODUCT(('资产主表'!$C$6:$C$242=A12)*(('资产主表'!$K$6:$K$242="已完成")+('资产主表'!$K$6:$K$242="原型已接入")+('资产主表'!$K$6:$K$242="正式美术已接入")+('资产主表'!$K$6:$K$242="已优化并正式接入")+('资产主表'!$K$6:$K$242="Blender源已完成")+('资产主表'!$K$6:$K$242="已导入；优化完成")+('资产主表'!$K$6:$K$242="白模源已完成；QA PASS")))</f>
+        <f>SUMPRODUCT(('资产主表'!$C$6:$C$246=A12)*(('资产主表'!$K$6:$K$246="已完成")+('资产主表'!$K$6:$K$246="原型已接入")+('资产主表'!$K$6:$K$246="正式美术已接入")+('资产主表'!$K$6:$K$246="已优化并正式接入")+('资产主表'!$K$6:$K$246="Blender源已完成")+('资产主表'!$K$6:$K$246="已导入；优化完成")+('资产主表'!$K$6:$K$246="白模源已完成；QA PASS")))</f>
         <v/>
       </c>
       <c r="D12" s="70" t="n"/>
@@ -1626,11 +1626,11 @@
         </is>
       </c>
       <c r="B13" s="66">
-        <f>COUNTIF('资产主表'!$C$6:$C$242,A13)</f>
+        <f>COUNTIF('资产主表'!$C$6:$C$246,A13)</f>
         <v/>
       </c>
       <c r="C13" s="66">
-        <f>SUMPRODUCT(('资产主表'!$C$6:$C$242=A13)*(('资产主表'!$K$6:$K$242="已完成")+('资产主表'!$K$6:$K$242="原型已接入")+('资产主表'!$K$6:$K$242="正式美术已接入")+('资产主表'!$K$6:$K$242="已优化并正式接入")+('资产主表'!$K$6:$K$242="Blender源已完成")+('资产主表'!$K$6:$K$242="已导入；优化完成")+('资产主表'!$K$6:$K$242="白模源已完成；QA PASS")))</f>
+        <f>SUMPRODUCT(('资产主表'!$C$6:$C$246=A13)*(('资产主表'!$K$6:$K$246="已完成")+('资产主表'!$K$6:$K$246="原型已接入")+('资产主表'!$K$6:$K$246="正式美术已接入")+('资产主表'!$K$6:$K$246="已优化并正式接入")+('资产主表'!$K$6:$K$246="Blender源已完成")+('资产主表'!$K$6:$K$246="已导入；优化完成")+('资产主表'!$K$6:$K$246="白模源已完成；QA PASS")))</f>
         <v/>
       </c>
       <c r="D13" s="66" t="n"/>
@@ -2194,7 +2194,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:Y242"/>
+  <dimension ref="A1:Y246"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.80859375" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="25" customWidth="1" style="59" min="1" max="1"/>
@@ -2470,7 +2470,7 @@
         <v/>
       </c>
       <c r="S6" s="71">
-        <f>IF(COUNTIF($R$6:$R$242,R6)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R6)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T6" s="71" t="n"/>
@@ -2577,7 +2577,7 @@
         <v/>
       </c>
       <c r="S7" s="71">
-        <f>IF(COUNTIF($R$6:$R$242,R7)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R7)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T7" s="71" t="n"/>
@@ -2684,7 +2684,7 @@
         <v/>
       </c>
       <c r="S8" s="71">
-        <f>IF(COUNTIF($R$6:$R$242,R8)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R8)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T8" s="71" t="n"/>
@@ -2791,7 +2791,7 @@
         <v/>
       </c>
       <c r="S9" s="71">
-        <f>IF(COUNTIF($R$6:$R$242,R9)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R9)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T9" s="71" t="n"/>
@@ -2898,7 +2898,7 @@
         <v/>
       </c>
       <c r="S10" s="71">
-        <f>IF(COUNTIF($R$6:$R$242,R10)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R10)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T10" s="71" t="n"/>
@@ -3005,7 +3005,7 @@
         <v/>
       </c>
       <c r="S11" s="71">
-        <f>IF(COUNTIF($R$6:$R$242,R11)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R11)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T11" s="71" t="n"/>
@@ -3112,7 +3112,7 @@
         <v/>
       </c>
       <c r="S12" s="71">
-        <f>IF(COUNTIF($R$6:$R$242,R12)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R12)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T12" s="71" t="n"/>
@@ -3219,7 +3219,7 @@
         <v/>
       </c>
       <c r="S13" s="71">
-        <f>IF(COUNTIF($R$6:$R$242,R13)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R13)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T13" s="71" t="n"/>
@@ -3326,7 +3326,7 @@
         <v/>
       </c>
       <c r="S14" s="71">
-        <f>IF(COUNTIF($R$6:$R$242,R14)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R14)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T14" s="71" t="n"/>
@@ -3433,7 +3433,7 @@
         <v/>
       </c>
       <c r="S15" s="71">
-        <f>IF(COUNTIF($R$6:$R$242,R15)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R15)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T15" s="71" t="n"/>
@@ -3540,7 +3540,7 @@
         <v/>
       </c>
       <c r="S16" s="71">
-        <f>IF(COUNTIF($R$6:$R$242,R16)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R16)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T16" s="71" t="n"/>
@@ -3647,7 +3647,7 @@
         <v/>
       </c>
       <c r="S17" s="71">
-        <f>IF(COUNTIF($R$6:$R$242,R17)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R17)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T17" s="71" t="n"/>
@@ -3754,7 +3754,7 @@
         <v/>
       </c>
       <c r="S18" s="71">
-        <f>IF(COUNTIF($R$6:$R$242,R18)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R18)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T18" s="71" t="n"/>
@@ -3861,7 +3861,7 @@
         <v/>
       </c>
       <c r="S19" s="71">
-        <f>IF(COUNTIF($R$6:$R$242,R19)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R19)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T19" s="71" t="n"/>
@@ -3968,7 +3968,7 @@
         <v/>
       </c>
       <c r="S20" s="71">
-        <f>IF(COUNTIF($R$6:$R$242,R20)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R20)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T20" s="71" t="n"/>
@@ -4075,7 +4075,7 @@
         <v/>
       </c>
       <c r="S21" s="71">
-        <f>IF(COUNTIF($R$6:$R$242,R21)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R21)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T21" s="71" t="n"/>
@@ -4182,7 +4182,7 @@
         <v/>
       </c>
       <c r="S22" s="71">
-        <f>IF(COUNTIF($R$6:$R$242,R22)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R22)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T22" s="71" t="n"/>
@@ -4289,7 +4289,7 @@
         <v/>
       </c>
       <c r="S23" s="71">
-        <f>IF(COUNTIF($R$6:$R$242,R23)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R23)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T23" s="71" t="n"/>
@@ -4396,7 +4396,7 @@
         <v/>
       </c>
       <c r="S24" s="71">
-        <f>IF(COUNTIF($R$6:$R$242,R24)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R24)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T24" s="71" t="n"/>
@@ -4503,7 +4503,7 @@
         <v/>
       </c>
       <c r="S25" s="71">
-        <f>IF(COUNTIF($R$6:$R$242,R25)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R25)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T25" s="71" t="n"/>
@@ -4610,7 +4610,7 @@
         <v/>
       </c>
       <c r="S26" s="71">
-        <f>IF(COUNTIF($R$6:$R$242,R26)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R26)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T26" s="71" t="n"/>
@@ -4717,7 +4717,7 @@
         <v/>
       </c>
       <c r="S27" s="71">
-        <f>IF(COUNTIF($R$6:$R$242,R27)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R27)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T27" s="71" t="n"/>
@@ -4824,7 +4824,7 @@
         <v/>
       </c>
       <c r="S28" s="71">
-        <f>IF(COUNTIF($R$6:$R$242,R28)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R28)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T28" s="71" t="n"/>
@@ -4931,7 +4931,7 @@
         <v/>
       </c>
       <c r="S29" s="71">
-        <f>IF(COUNTIF($R$6:$R$242,R29)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R29)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T29" s="71" t="n"/>
@@ -5038,7 +5038,7 @@
         <v/>
       </c>
       <c r="S30" s="71">
-        <f>IF(COUNTIF($R$6:$R$242,R30)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R30)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T30" s="71" t="n"/>
@@ -5145,7 +5145,7 @@
         <v/>
       </c>
       <c r="S31" s="71">
-        <f>IF(COUNTIF($R$6:$R$242,R31)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R31)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T31" s="71" t="n"/>
@@ -5264,7 +5264,7 @@
         <v/>
       </c>
       <c r="S32" s="88">
-        <f>IF(COUNTIF($R$6:$R$242,R32)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R32)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T32" s="87" t="inlineStr">
@@ -5387,7 +5387,7 @@
         <v/>
       </c>
       <c r="S33" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R33)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R33)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T33" s="90" t="inlineStr">
@@ -5510,7 +5510,7 @@
         <v/>
       </c>
       <c r="S34" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R34)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R34)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T34" s="90" t="inlineStr">
@@ -5633,7 +5633,7 @@
         <v/>
       </c>
       <c r="S35" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R35)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R35)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T35" s="90" t="inlineStr">
@@ -5756,7 +5756,7 @@
         <v/>
       </c>
       <c r="S36" s="88">
-        <f>IF(COUNTIF($R$6:$R$242,R36)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R36)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T36" s="87" t="inlineStr">
@@ -5880,7 +5880,7 @@
         <v/>
       </c>
       <c r="S37" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R37)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R37)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T37" s="90" t="inlineStr">
@@ -6003,7 +6003,7 @@
         <v/>
       </c>
       <c r="S38" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R38)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R38)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T38" s="90" t="inlineStr">
@@ -6122,7 +6122,7 @@
         <v/>
       </c>
       <c r="S39" s="88">
-        <f>IF(COUNTIF($R$6:$R$242,R39)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R39)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T39" s="87" t="inlineStr">
@@ -6245,7 +6245,7 @@
         <v/>
       </c>
       <c r="S40" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R40)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R40)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T40" s="90" t="inlineStr">
@@ -6368,7 +6368,7 @@
         <v/>
       </c>
       <c r="S41" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R41)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R41)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T41" s="90" t="inlineStr">
@@ -6491,7 +6491,7 @@
         <v/>
       </c>
       <c r="S42" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R42)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R42)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T42" s="90" t="inlineStr">
@@ -6614,7 +6614,7 @@
         <v/>
       </c>
       <c r="S43" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R43)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R43)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T43" s="90" t="inlineStr">
@@ -6737,7 +6737,7 @@
         <v/>
       </c>
       <c r="S44" s="88">
-        <f>IF(COUNTIF($R$6:$R$242,R44)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R44)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T44" s="87" t="inlineStr">
@@ -6861,7 +6861,7 @@
         <v/>
       </c>
       <c r="S45" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R45)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R45)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T45" s="90" t="inlineStr">
@@ -6984,7 +6984,7 @@
         <v/>
       </c>
       <c r="S46" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R46)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R46)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T46" s="90" t="inlineStr">
@@ -7107,7 +7107,7 @@
         <v/>
       </c>
       <c r="S47" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R47)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R47)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T47" s="90" t="inlineStr">
@@ -7230,7 +7230,7 @@
         <v/>
       </c>
       <c r="S48" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R48)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R48)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T48" s="90" t="inlineStr">
@@ -7350,7 +7350,7 @@
         <v/>
       </c>
       <c r="S49" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R49)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R49)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T49" s="90" t="inlineStr">
@@ -7473,7 +7473,7 @@
         <v/>
       </c>
       <c r="S50" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R50)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R50)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T50" s="90" t="inlineStr">
@@ -7597,7 +7597,7 @@
         <v/>
       </c>
       <c r="S51" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R51)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R51)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T51" s="90" t="inlineStr">
@@ -7720,7 +7720,7 @@
         <v/>
       </c>
       <c r="S52" s="88">
-        <f>IF(COUNTIF($R$6:$R$242,R52)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R52)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T52" s="87" t="inlineStr">
@@ -7844,7 +7844,7 @@
         <v/>
       </c>
       <c r="S53" s="88">
-        <f>IF(COUNTIF($R$6:$R$242,R53)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R53)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T53" s="87" t="inlineStr">
@@ -7967,7 +7967,7 @@
         <v/>
       </c>
       <c r="S54" s="88">
-        <f>IF(COUNTIF($R$6:$R$242,R54)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R54)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T54" s="87" t="inlineStr">
@@ -8096,7 +8096,7 @@
         <v/>
       </c>
       <c r="S55" s="88">
-        <f>IF(COUNTIF($R$6:$R$242,R55)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R55)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T55" s="87" t="inlineStr">
@@ -8223,7 +8223,7 @@
         <v/>
       </c>
       <c r="S56" s="88">
-        <f>IF(COUNTIF($R$6:$R$242,R56)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R56)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T56" s="87" t="inlineStr">
@@ -8346,7 +8346,7 @@
         <v/>
       </c>
       <c r="S57" s="88">
-        <f>IF(COUNTIF($R$6:$R$242,R57)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R57)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T57" s="87" t="inlineStr">
@@ -8471,7 +8471,7 @@
         <v/>
       </c>
       <c r="S58" s="88">
-        <f>IF(COUNTIF($R$6:$R$242,R58)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R58)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T58" s="87" t="inlineStr">
@@ -8594,7 +8594,7 @@
         <v/>
       </c>
       <c r="S59" s="88">
-        <f>IF(COUNTIF($R$6:$R$242,R59)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R59)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T59" s="87" t="inlineStr">
@@ -8713,7 +8713,7 @@
         <v/>
       </c>
       <c r="S60" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R60)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R60)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T60" s="90" t="inlineStr">
@@ -8833,7 +8833,7 @@
         <v/>
       </c>
       <c r="S61" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R61)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R61)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T61" s="90" t="inlineStr">
@@ -8953,7 +8953,7 @@
         <v/>
       </c>
       <c r="S62" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R62)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R62)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T62" s="90" t="inlineStr">
@@ -9073,7 +9073,7 @@
         <v/>
       </c>
       <c r="S63" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R63)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R63)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T63" s="90" t="n"/>
@@ -9193,7 +9193,7 @@
         <v/>
       </c>
       <c r="S64" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R64)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R64)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T64" s="90" t="inlineStr">
@@ -9318,7 +9318,7 @@
         <v/>
       </c>
       <c r="S65" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R65)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R65)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T65" s="90" t="inlineStr">
@@ -9443,7 +9443,7 @@
         <v/>
       </c>
       <c r="S66" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R66)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R66)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T66" s="90" t="inlineStr">
@@ -9568,7 +9568,7 @@
         <v/>
       </c>
       <c r="S67" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R67)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R67)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T67" s="90" t="inlineStr">
@@ -9693,7 +9693,7 @@
         <v/>
       </c>
       <c r="S68" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R68)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R68)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T68" s="90" t="inlineStr">
@@ -9824,7 +9824,7 @@
         <v/>
       </c>
       <c r="S69" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R69)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R69)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T69" s="90" t="inlineStr">
@@ -9950,7 +9950,7 @@
         <v/>
       </c>
       <c r="S70" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R70)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R70)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T70" s="90" t="inlineStr">
@@ -10074,7 +10074,7 @@
         <v/>
       </c>
       <c r="S71" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R71)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R71)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T71" s="90" t="inlineStr">
@@ -10198,7 +10198,7 @@
         <v/>
       </c>
       <c r="S72" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R72)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R72)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T72" s="90" t="inlineStr">
@@ -10322,7 +10322,7 @@
         <v/>
       </c>
       <c r="S73" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R73)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R73)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T73" s="90" t="inlineStr">
@@ -10446,7 +10446,7 @@
         <v/>
       </c>
       <c r="S74" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R74)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R74)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T74" s="90" t="inlineStr">
@@ -10570,7 +10570,7 @@
         <v/>
       </c>
       <c r="S75" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R75)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R75)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T75" s="90" t="inlineStr">
@@ -10694,7 +10694,7 @@
         <v/>
       </c>
       <c r="S76" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R76)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R76)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T76" s="90" t="inlineStr">
@@ -10818,7 +10818,7 @@
         <v/>
       </c>
       <c r="S77" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R77)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R77)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T77" s="90" t="inlineStr">
@@ -10942,7 +10942,7 @@
         <v/>
       </c>
       <c r="S78" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R78)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R78)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T78" s="90" t="inlineStr">
@@ -11066,7 +11066,7 @@
         <v/>
       </c>
       <c r="S79" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R79)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R79)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T79" s="90" t="inlineStr">
@@ -11190,7 +11190,7 @@
         <v/>
       </c>
       <c r="S80" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R80)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R80)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T80" s="90" t="inlineStr">
@@ -11314,7 +11314,7 @@
         <v/>
       </c>
       <c r="S81" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R81)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R81)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T81" s="90" t="inlineStr">
@@ -11438,7 +11438,7 @@
         <v/>
       </c>
       <c r="S82" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R82)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R82)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T82" s="90" t="inlineStr">
@@ -11562,7 +11562,7 @@
         <v/>
       </c>
       <c r="S83" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R83)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R83)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T83" s="90" t="inlineStr">
@@ -11686,7 +11686,7 @@
         <v/>
       </c>
       <c r="S84" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R84)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R84)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T84" s="90" t="inlineStr">
@@ -11810,7 +11810,7 @@
         <v/>
       </c>
       <c r="S85" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R85)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R85)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T85" s="90" t="inlineStr">
@@ -11934,7 +11934,7 @@
         <v/>
       </c>
       <c r="S86" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R86)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R86)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T86" s="90" t="inlineStr">
@@ -12058,7 +12058,7 @@
         <v/>
       </c>
       <c r="S87" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R87)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R87)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T87" s="90" t="inlineStr">
@@ -12182,7 +12182,7 @@
         <v/>
       </c>
       <c r="S88" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R88)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R88)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T88" s="90" t="inlineStr">
@@ -12306,7 +12306,7 @@
         <v/>
       </c>
       <c r="S89" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R89)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R89)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T89" s="90" t="inlineStr">
@@ -12430,7 +12430,7 @@
         <v/>
       </c>
       <c r="S90" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R90)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R90)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T90" s="90" t="inlineStr">
@@ -12554,7 +12554,7 @@
         <v/>
       </c>
       <c r="S91" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R91)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R91)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T91" s="90" t="inlineStr">
@@ -12678,7 +12678,7 @@
         <v/>
       </c>
       <c r="S92" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R92)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R92)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T92" s="90" t="inlineStr">
@@ -12802,7 +12802,7 @@
         <v/>
       </c>
       <c r="S93" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R93)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R93)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T93" s="90" t="inlineStr">
@@ -12926,7 +12926,7 @@
         <v/>
       </c>
       <c r="S94" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R94)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R94)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T94" s="90" t="inlineStr">
@@ -13050,7 +13050,7 @@
         <v/>
       </c>
       <c r="S95" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R95)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R95)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T95" s="90" t="inlineStr">
@@ -13174,7 +13174,7 @@
         <v/>
       </c>
       <c r="S96" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R96)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R96)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T96" s="90" t="inlineStr">
@@ -13298,7 +13298,7 @@
         <v/>
       </c>
       <c r="S97" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R97)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R97)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T97" s="90" t="inlineStr">
@@ -13422,7 +13422,7 @@
         <v/>
       </c>
       <c r="S98" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R98)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R98)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T98" s="90" t="inlineStr">
@@ -13546,7 +13546,7 @@
         <v/>
       </c>
       <c r="S99" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R99)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R99)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T99" s="90" t="inlineStr">
@@ -13670,7 +13670,7 @@
         <v/>
       </c>
       <c r="S100" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R100)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R100)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T100" s="90" t="inlineStr">
@@ -13794,7 +13794,7 @@
         <v/>
       </c>
       <c r="S101" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R101)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R101)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T101" s="90" t="inlineStr">
@@ -13918,7 +13918,7 @@
         <v/>
       </c>
       <c r="S102" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R102)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R102)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T102" s="90" t="inlineStr">
@@ -14041,7 +14041,7 @@
         <v/>
       </c>
       <c r="S103" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R103)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R103)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T103" s="90" t="inlineStr">
@@ -14166,7 +14166,7 @@
         <v/>
       </c>
       <c r="S104" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R104)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R104)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T104" s="90" t="inlineStr">
@@ -14291,7 +14291,7 @@
         <v/>
       </c>
       <c r="S105" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R105)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R105)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T105" s="90" t="inlineStr">
@@ -14416,7 +14416,7 @@
         <v/>
       </c>
       <c r="S106" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R106)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R106)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T106" s="90" t="inlineStr">
@@ -14541,7 +14541,7 @@
         <v/>
       </c>
       <c r="S107" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R107)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R107)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T107" s="90" t="inlineStr">
@@ -14666,7 +14666,7 @@
         <v/>
       </c>
       <c r="S108" s="94">
-        <f>IF(COUNTIF($R$6:$R$242,R108)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R108)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T108" s="93" t="inlineStr">
@@ -14792,7 +14792,7 @@
         <v/>
       </c>
       <c r="S109" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R109)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R109)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T109" s="90" t="inlineStr">
@@ -14918,7 +14918,7 @@
         <v/>
       </c>
       <c r="S110" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R110)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R110)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T110" s="90" t="inlineStr">
@@ -15044,7 +15044,7 @@
         <v/>
       </c>
       <c r="S111" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R111)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R111)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T111" s="90" t="inlineStr">
@@ -15170,7 +15170,7 @@
         <v/>
       </c>
       <c r="S112" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R112)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R112)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T112" s="90" t="inlineStr">
@@ -15293,7 +15293,7 @@
         <v/>
       </c>
       <c r="S113" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R113)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R113)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T113" s="90" t="inlineStr">
@@ -15413,7 +15413,7 @@
         <v/>
       </c>
       <c r="S114" s="94">
-        <f>IF(COUNTIF($R$6:$R$242,R114)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R114)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T114" s="93" t="inlineStr">
@@ -15532,7 +15532,7 @@
         <v/>
       </c>
       <c r="S115" s="94">
-        <f>IF(COUNTIF($R$6:$R$242,R115)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R115)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T115" s="93" t="inlineStr">
@@ -15650,7 +15650,7 @@
         <v/>
       </c>
       <c r="S116" s="94">
-        <f>IF(COUNTIF($R$6:$R$242,R116)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R116)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T116" s="93" t="inlineStr">
@@ -15773,7 +15773,7 @@
         <v/>
       </c>
       <c r="S117" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R117)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R117)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T117" s="90" t="inlineStr">
@@ -15899,7 +15899,7 @@
         <v/>
       </c>
       <c r="S118" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R118)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R118)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T118" s="90" t="inlineStr">
@@ -16022,7 +16022,7 @@
         <v/>
       </c>
       <c r="S119" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R119)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R119)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T119" s="90" t="inlineStr">
@@ -16147,7 +16147,7 @@
         <v/>
       </c>
       <c r="S120" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R120)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R120)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T120" s="90" t="inlineStr">
@@ -16270,7 +16270,7 @@
         <v/>
       </c>
       <c r="S121" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R121)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R121)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T121" s="90" t="inlineStr">
@@ -16395,7 +16395,7 @@
         <v/>
       </c>
       <c r="S122" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R122)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R122)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T122" s="90" t="inlineStr">
@@ -16518,7 +16518,7 @@
         <v/>
       </c>
       <c r="S123" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R123)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R123)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T123" s="90" t="inlineStr">
@@ -16641,7 +16641,7 @@
         <v/>
       </c>
       <c r="S124" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R124)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R124)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T124" s="90" t="inlineStr">
@@ -16764,7 +16764,7 @@
         <v/>
       </c>
       <c r="S125" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R125)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R125)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T125" s="90" t="inlineStr">
@@ -16887,7 +16887,7 @@
         <v/>
       </c>
       <c r="S126" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R126)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R126)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T126" s="90" t="inlineStr">
@@ -17010,7 +17010,7 @@
         <v/>
       </c>
       <c r="S127" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R127)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R127)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T127" s="90" t="inlineStr">
@@ -17133,7 +17133,7 @@
         <v/>
       </c>
       <c r="S128" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R128)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R128)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T128" s="90" t="inlineStr">
@@ -17256,7 +17256,7 @@
         <v/>
       </c>
       <c r="S129" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R129)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R129)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T129" s="90" t="inlineStr">
@@ -17379,7 +17379,7 @@
         <v/>
       </c>
       <c r="S130" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R130)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R130)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T130" s="90" t="inlineStr">
@@ -17502,7 +17502,7 @@
         <v/>
       </c>
       <c r="S131" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R131)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R131)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T131" s="90" t="inlineStr">
@@ -17625,7 +17625,7 @@
         <v/>
       </c>
       <c r="S132" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R132)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R132)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T132" s="90" t="inlineStr">
@@ -17749,7 +17749,7 @@
         <v/>
       </c>
       <c r="S133" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R133)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R133)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T133" s="90" t="inlineStr">
@@ -17872,7 +17872,7 @@
         <v/>
       </c>
       <c r="S134" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R134)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R134)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T134" s="90" t="inlineStr">
@@ -17995,7 +17995,7 @@
         <v/>
       </c>
       <c r="S135" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R135)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R135)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T135" s="90" t="inlineStr">
@@ -18121,7 +18121,7 @@
         <v/>
       </c>
       <c r="S136" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R136)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R136)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T136" s="90" t="inlineStr">
@@ -18247,7 +18247,7 @@
         <v/>
       </c>
       <c r="S137" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R137)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R137)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T137" s="90" t="inlineStr">
@@ -18373,7 +18373,7 @@
         <v/>
       </c>
       <c r="S138" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R138)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R138)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T138" s="90" t="inlineStr">
@@ -18499,7 +18499,7 @@
         <v/>
       </c>
       <c r="S139" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R139)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R139)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T139" s="90" t="inlineStr">
@@ -18625,7 +18625,7 @@
         <v/>
       </c>
       <c r="S140" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R140)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R140)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T140" s="90" t="inlineStr">
@@ -18751,7 +18751,7 @@
         <v/>
       </c>
       <c r="S141" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R141)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R141)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T141" s="90" t="inlineStr">
@@ -18877,7 +18877,7 @@
         <v/>
       </c>
       <c r="S142" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R142)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R142)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T142" s="90" t="inlineStr">
@@ -19003,7 +19003,7 @@
         <v/>
       </c>
       <c r="S143" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R143)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R143)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T143" s="90" t="inlineStr">
@@ -19129,7 +19129,7 @@
         <v/>
       </c>
       <c r="S144" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R144)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R144)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T144" s="90" t="inlineStr">
@@ -19255,7 +19255,7 @@
         <v/>
       </c>
       <c r="S145" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R145)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R145)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T145" s="90" t="inlineStr">
@@ -19381,7 +19381,7 @@
         <v/>
       </c>
       <c r="S146" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R146)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R146)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T146" s="90" t="inlineStr">
@@ -19507,7 +19507,7 @@
         <v/>
       </c>
       <c r="S147" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R147)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R147)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T147" s="90" t="inlineStr">
@@ -19633,7 +19633,7 @@
         <v/>
       </c>
       <c r="S148" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R148)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R148)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T148" s="90" t="inlineStr">
@@ -19759,7 +19759,7 @@
         <v/>
       </c>
       <c r="S149" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R149)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R149)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T149" s="90" t="inlineStr">
@@ -19885,7 +19885,7 @@
         <v/>
       </c>
       <c r="S150" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R150)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R150)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T150" s="90" t="inlineStr">
@@ -20011,7 +20011,7 @@
         <v/>
       </c>
       <c r="S151" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R151)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R151)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T151" s="90" t="inlineStr">
@@ -20137,7 +20137,7 @@
         <v/>
       </c>
       <c r="S152" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R152)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R152)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T152" s="90" t="inlineStr">
@@ -20263,7 +20263,7 @@
         <v/>
       </c>
       <c r="S153" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R153)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R153)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T153" s="90" t="inlineStr">
@@ -20389,7 +20389,7 @@
         <v/>
       </c>
       <c r="S154" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R154)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R154)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T154" s="90" t="inlineStr">
@@ -20515,7 +20515,7 @@
         <v/>
       </c>
       <c r="S155" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R155)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R155)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T155" s="90" t="inlineStr">
@@ -20641,7 +20641,7 @@
         <v/>
       </c>
       <c r="S156" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R156)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R156)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T156" s="90" t="inlineStr">
@@ -20767,7 +20767,7 @@
         <v/>
       </c>
       <c r="S157" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R157)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R157)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T157" s="90" t="inlineStr">
@@ -20893,7 +20893,7 @@
         <v/>
       </c>
       <c r="S158" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R158)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R158)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T158" s="90" t="inlineStr">
@@ -21019,7 +21019,7 @@
         <v/>
       </c>
       <c r="S159" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R159)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R159)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T159" s="90" t="inlineStr">
@@ -21145,7 +21145,7 @@
         <v/>
       </c>
       <c r="S160" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R160)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R160)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T160" s="90" t="inlineStr">
@@ -21271,7 +21271,7 @@
         <v/>
       </c>
       <c r="S161" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R161)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R161)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T161" s="90" t="inlineStr">
@@ -21397,7 +21397,7 @@
         <v/>
       </c>
       <c r="S162" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R162)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R162)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T162" s="90" t="inlineStr">
@@ -21523,7 +21523,7 @@
         <v/>
       </c>
       <c r="S163" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R163)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R163)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T163" s="90" t="inlineStr">
@@ -21649,7 +21649,7 @@
         <v/>
       </c>
       <c r="S164" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R164)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R164)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T164" s="90" t="inlineStr">
@@ -21775,7 +21775,7 @@
         <v/>
       </c>
       <c r="S165" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R165)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R165)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T165" s="90" t="inlineStr">
@@ -21901,7 +21901,7 @@
         <v/>
       </c>
       <c r="S166" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R166)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R166)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T166" s="90" t="inlineStr">
@@ -22027,7 +22027,7 @@
         <v/>
       </c>
       <c r="S167" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R167)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R167)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T167" s="90" t="inlineStr">
@@ -22153,7 +22153,7 @@
         <v/>
       </c>
       <c r="S168" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R168)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R168)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T168" s="90" t="inlineStr">
@@ -22279,7 +22279,7 @@
         <v/>
       </c>
       <c r="S169" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R169)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R169)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T169" s="90" t="inlineStr">
@@ -22405,7 +22405,7 @@
         <v/>
       </c>
       <c r="S170" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R170)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R170)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T170" s="90" t="inlineStr">
@@ -22531,7 +22531,7 @@
         <v/>
       </c>
       <c r="S171" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R171)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R171)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T171" s="90" t="inlineStr">
@@ -22654,7 +22654,7 @@
         <v/>
       </c>
       <c r="S172" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R172)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R172)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T172" s="90" t="inlineStr">
@@ -22777,7 +22777,7 @@
         <v/>
       </c>
       <c r="S173" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R173)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R173)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T173" s="90" t="inlineStr">
@@ -22901,7 +22901,7 @@
         <v/>
       </c>
       <c r="S174" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R174)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R174)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T174" s="90" t="inlineStr">
@@ -23025,7 +23025,7 @@
         <v/>
       </c>
       <c r="S175" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R175)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R175)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T175" s="90" t="inlineStr">
@@ -23149,7 +23149,7 @@
         <v/>
       </c>
       <c r="S176" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R176)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R176)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T176" s="90" t="inlineStr">
@@ -23273,7 +23273,7 @@
         <v/>
       </c>
       <c r="S177" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R177)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R177)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T177" s="90" t="inlineStr">
@@ -23397,7 +23397,7 @@
         <v/>
       </c>
       <c r="S178" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R178)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R178)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T178" s="90" t="inlineStr">
@@ -23522,7 +23522,7 @@
         <v/>
       </c>
       <c r="S179" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R179)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R179)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T179" s="90" t="inlineStr">
@@ -23645,7 +23645,7 @@
         <v/>
       </c>
       <c r="S180" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R180)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R180)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T180" s="90" t="inlineStr">
@@ -23769,7 +23769,7 @@
         <v/>
       </c>
       <c r="S181" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R181)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R181)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T181" s="90" t="inlineStr">
@@ -23892,7 +23892,7 @@
         <v/>
       </c>
       <c r="S182" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R182)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R182)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T182" s="90" t="inlineStr">
@@ -24015,7 +24015,7 @@
         <v/>
       </c>
       <c r="S183" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R183)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R183)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T183" s="90" t="inlineStr">
@@ -24139,7 +24139,7 @@
         <v/>
       </c>
       <c r="S184" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R184)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R184)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T184" s="90" t="inlineStr">
@@ -24264,7 +24264,7 @@
         <v/>
       </c>
       <c r="S185" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R185)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R185)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T185" s="90" t="inlineStr">
@@ -24388,7 +24388,7 @@
         <v/>
       </c>
       <c r="S186" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R186)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R186)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T186" s="90" t="inlineStr">
@@ -24512,7 +24512,7 @@
         <v/>
       </c>
       <c r="S187" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R187)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R187)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T187" s="90" t="inlineStr">
@@ -24636,7 +24636,7 @@
         <v/>
       </c>
       <c r="S188" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R188)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R188)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T188" s="90" t="inlineStr">
@@ -24760,7 +24760,7 @@
         <v/>
       </c>
       <c r="S189" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R189)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R189)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T189" s="90" t="inlineStr">
@@ -24884,7 +24884,7 @@
         <v/>
       </c>
       <c r="S190" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R190)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R190)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T190" s="90" t="inlineStr">
@@ -25008,7 +25008,7 @@
         <v/>
       </c>
       <c r="S191" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R191)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R191)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T191" s="90" t="inlineStr">
@@ -25131,7 +25131,7 @@
         <v/>
       </c>
       <c r="S192" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R192)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R192)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T192" s="90" t="inlineStr">
@@ -25255,7 +25255,7 @@
         <v/>
       </c>
       <c r="S193" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R193)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R193)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T193" s="90" t="inlineStr">
@@ -25378,7 +25378,7 @@
         <v/>
       </c>
       <c r="S194" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R194)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R194)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T194" s="90" t="inlineStr">
@@ -25501,7 +25501,7 @@
         <v/>
       </c>
       <c r="S195" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R195)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R195)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T195" s="90" t="inlineStr">
@@ -25625,7 +25625,7 @@
         <v/>
       </c>
       <c r="S196" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R196)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R196)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T196" s="90" t="inlineStr">
@@ -25748,7 +25748,7 @@
         <v/>
       </c>
       <c r="S197" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R197)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R197)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T197" s="90" t="inlineStr">
@@ -25871,7 +25871,7 @@
         <v/>
       </c>
       <c r="S198" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R198)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R198)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T198" s="90" t="inlineStr">
@@ -25994,7 +25994,7 @@
         <v/>
       </c>
       <c r="S199" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R199)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R199)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T199" s="90" t="inlineStr">
@@ -26117,7 +26117,7 @@
         <v/>
       </c>
       <c r="S200" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R200)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R200)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T200" s="90" t="inlineStr">
@@ -26240,7 +26240,7 @@
         <v/>
       </c>
       <c r="S201" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R201)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R201)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T201" s="90" t="inlineStr">
@@ -26363,7 +26363,7 @@
         <v/>
       </c>
       <c r="S202" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R202)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R202)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T202" s="90" t="inlineStr">
@@ -26486,7 +26486,7 @@
         <v/>
       </c>
       <c r="S203" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R203)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R203)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T203" s="90" t="inlineStr">
@@ -26609,7 +26609,7 @@
         <v/>
       </c>
       <c r="S204" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R204)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R204)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T204" s="90" t="inlineStr">
@@ -26733,7 +26733,7 @@
         <v/>
       </c>
       <c r="S205" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R205)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R205)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T205" s="90" t="inlineStr">
@@ -26857,7 +26857,7 @@
         <v/>
       </c>
       <c r="S206" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R206)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R206)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T206" s="90" t="inlineStr">
@@ -26980,7 +26980,7 @@
         <v/>
       </c>
       <c r="S207" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R207)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R207)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T207" s="90" t="inlineStr">
@@ -27103,7 +27103,7 @@
         <v/>
       </c>
       <c r="S208" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R208)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R208)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T208" s="90" t="inlineStr">
@@ -27226,7 +27226,7 @@
         <v/>
       </c>
       <c r="S209" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R209)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R209)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T209" s="90" t="inlineStr">
@@ -27349,7 +27349,7 @@
         <v/>
       </c>
       <c r="S210" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R210)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R210)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T210" s="90" t="inlineStr">
@@ -27472,7 +27472,7 @@
         <v/>
       </c>
       <c r="S211" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R211)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R211)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T211" s="90" t="inlineStr">
@@ -27595,7 +27595,7 @@
         <v/>
       </c>
       <c r="S212" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R212)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R212)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T212" s="90" t="inlineStr">
@@ -27718,7 +27718,7 @@
         <v/>
       </c>
       <c r="S213" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R213)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R213)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T213" s="90" t="inlineStr">
@@ -27841,7 +27841,7 @@
         <v/>
       </c>
       <c r="S214" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R214)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R214)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T214" s="90" t="inlineStr">
@@ -27964,7 +27964,7 @@
         <v/>
       </c>
       <c r="S215" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R215)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R215)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T215" s="90" t="inlineStr">
@@ -28087,7 +28087,7 @@
         <v/>
       </c>
       <c r="S216" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R216)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R216)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T216" s="90" t="inlineStr">
@@ -28210,7 +28210,7 @@
         <v/>
       </c>
       <c r="S217" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R217)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R217)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T217" s="90" t="inlineStr">
@@ -28334,7 +28334,7 @@
         <v/>
       </c>
       <c r="S218" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R218)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R218)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T218" s="90" t="inlineStr">
@@ -28457,7 +28457,7 @@
         <v/>
       </c>
       <c r="S219" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R219)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R219)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T219" s="90" t="inlineStr">
@@ -28580,7 +28580,7 @@
         <v/>
       </c>
       <c r="S220" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R220)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R220)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T220" s="90" t="inlineStr">
@@ -28703,7 +28703,7 @@
         <v/>
       </c>
       <c r="S221" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R221)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R221)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T221" s="90" t="inlineStr">
@@ -28826,7 +28826,7 @@
         <v/>
       </c>
       <c r="S222" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R222)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R222)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T222" s="90" t="inlineStr">
@@ -28949,7 +28949,7 @@
         <v/>
       </c>
       <c r="S223" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R223)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R223)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T223" s="90" t="inlineStr">
@@ -29072,7 +29072,7 @@
         <v/>
       </c>
       <c r="S224" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R224)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R224)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T224" s="90" t="inlineStr">
@@ -29195,7 +29195,7 @@
         <v/>
       </c>
       <c r="S225" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R225)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R225)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T225" s="90" t="inlineStr">
@@ -29318,7 +29318,7 @@
         <v/>
       </c>
       <c r="S226" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R226)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R226)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T226" s="90" t="inlineStr">
@@ -29441,7 +29441,7 @@
         <v/>
       </c>
       <c r="S227" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R227)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R227)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T227" s="90" t="inlineStr">
@@ -29564,7 +29564,7 @@
         <v/>
       </c>
       <c r="S228" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R228)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R228)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T228" s="90" t="inlineStr">
@@ -29687,7 +29687,7 @@
         <v/>
       </c>
       <c r="S229" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R229)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R229)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T229" s="90" t="inlineStr">
@@ -29810,7 +29810,7 @@
         <v/>
       </c>
       <c r="S230" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R230)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R230)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T230" s="90" t="inlineStr">
@@ -29934,7 +29934,7 @@
         <v/>
       </c>
       <c r="S231" s="94">
-        <f>IF(COUNTIF($R$6:$R$242,R231)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R231)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T231" s="93" t="inlineStr">
@@ -30057,7 +30057,7 @@
         <v/>
       </c>
       <c r="S232" s="94">
-        <f>IF(COUNTIF($R$6:$R$242,R232)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R232)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T232" s="93" t="inlineStr">
@@ -30177,7 +30177,7 @@
         <v/>
       </c>
       <c r="S233" s="94">
-        <f>IF(COUNTIF($R$6:$R$242,R233)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R233)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="U233" s="93" t="inlineStr">
@@ -30293,7 +30293,7 @@
         <v/>
       </c>
       <c r="S234" s="94">
-        <f>IF(COUNTIF($R$6:$R$242,R234)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R234)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="U234" s="93" t="inlineStr">
@@ -30409,7 +30409,7 @@
         <v/>
       </c>
       <c r="S235" s="94">
-        <f>IF(COUNTIF($R$6:$R$242,R235)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R235)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="U235" s="93" t="inlineStr">
@@ -30525,7 +30525,7 @@
         <v/>
       </c>
       <c r="S236" s="94">
-        <f>IF(COUNTIF($R$6:$R$242,R236)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R236)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="U236" s="93" t="inlineStr">
@@ -30641,7 +30641,7 @@
         <v/>
       </c>
       <c r="S237" s="94">
-        <f>IF(COUNTIF($R$6:$R$242,R237)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R237)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="U237" s="93" t="inlineStr">
@@ -30758,7 +30758,7 @@
         <v/>
       </c>
       <c r="S238" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R238)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R238)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T238" s="90" t="inlineStr">
@@ -30881,7 +30881,7 @@
         <v/>
       </c>
       <c r="S239" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R239)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R239)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T239" s="90" t="inlineStr">
@@ -31000,7 +31000,7 @@
         <v/>
       </c>
       <c r="S240" s="63">
-        <f>IF(COUNTIF($R$6:$R$242,R240)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R240)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T240" s="90" t="inlineStr">
@@ -31119,7 +31119,7 @@
         <v/>
       </c>
       <c r="S241" s="90">
-        <f>IF(COUNTIF($R$6:$R$242,R241)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R241)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T241" s="90" t="inlineStr">
@@ -31240,7 +31240,7 @@
         <v/>
       </c>
       <c r="S242" s="90">
-        <f>IF(COUNTIF($R$6:$R$242,R242)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$246,R242)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T242" s="90" t="inlineStr">
@@ -31271,6 +31271,490 @@
       <c r="Y242" s="63" t="inlineStr">
         <is>
           <t>由 battle 区块房间种类源迁入（原 ENV-BATTLE-L-CORRIDOR-TYPE，原路径 tower_zones/battle/source/room_types/l_corridor/；业主 2026-09-24 裁决归属远征关卡01，battle 侧不留副本）。远征01 版图与白盒目录均无走廊白模，尺寸与门位按参考图推定。v001/v002 为 10m 宽走廊（外包络 45×35m / 28 块地砖 / 88、111 个组件包），v003 拓宽为 15m（45×40m / 42 块地砖 / 121 个组件包 / 4 个门位：西1 北2 南1）。随迁统一内部结构：component_packages_vNNN→component_packages、facility→facilities、散放渲染图入 renders/。共享件引用由 ENV-BATTLE-COMMON-* 更正为 shared 库现有 ENV-SHARED-GENERIC-*。未导 GLB、未接 Godot。</t>
+        </is>
+      </c>
+    </row>
+    <row r="243" ht="255" customHeight="1" s="60">
+      <c r="A243" s="90" t="inlineStr">
+        <is>
+          <t>ENV-EXPEDITION-L01-OFFICE-ROOM</t>
+        </is>
+      </c>
+      <c r="B243" s="63" t="inlineStr">
+        <is>
+          <t>远征关卡01 办公室 开放办公 30×40m 房间种类源</t>
+        </is>
+      </c>
+      <c r="C243" s="63" t="inlineStr">
+        <is>
+          <t>场景</t>
+        </is>
+      </c>
+      <c r="D243" s="90" t="inlineStr">
+        <is>
+          <t>office_room</t>
+        </is>
+      </c>
+      <c r="E243" s="90" t="inlineStr">
+        <is>
+          <t>expedition_01_office_room</t>
+        </is>
+      </c>
+      <c r="F243" s="90" t="inlineStr">
+        <is>
+          <t>room_type</t>
+        </is>
+      </c>
+      <c r="G243" s="90" t="n"/>
+      <c r="H243" s="90" t="inlineStr">
+        <is>
+          <t>Top3D / Blender Z-up</t>
+        </is>
+      </c>
+      <c r="I243" s="90" t="inlineStr">
+        <is>
+          <t>scene_art / reference_derived</t>
+        </is>
+      </c>
+      <c r="J243" s="63" t="inlineStr">
+        <is>
+          <t>远征关卡01 专用；room_03 与 room_09 两处实例共用同一房型源（同 office_60x70 模板）</t>
+        </is>
+      </c>
+      <c r="K243" s="90" t="inlineStr">
+        <is>
+          <t>Blender源已完成</t>
+        </is>
+      </c>
+      <c r="L243" s="90" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="M243" s="90" t="inlineStr">
+        <is>
+          <t>v001</t>
+        </is>
+      </c>
+      <c r="N243" s="90" t="inlineStr">
+        <is>
+          <t>30×40×11.9m（6×8 个 5m 槽 / 28 个墙位）；106 个独立组件包 / 193 输出网格 / 211708 面；无内墙；4 组工位；门洞 2.2×2.5m（净空底 0.30m、门楣 2.80m）；QA PASS（22 项断言）</t>
+        </is>
+      </c>
+      <c r="O243" s="90" t="inlineStr">
+        <is>
+          <t>assets/art/environments/tower_zones/expedition/source/room_types/office_room/v001/办公室房间种类_开放办公_30x40m_v001.blend</t>
+        </is>
+      </c>
+      <c r="P243" s="90" t="inlineStr">
+        <is>
+          <t>assets/art/environments/tower_zones/expedition/source/room_types/office_room/v001/build_office_room_v001.py；白盒 source/art/whitebox/tower_zones/expedition_01/v001/data/room_templates/office_60x70.json</t>
+        </is>
+      </c>
+      <c r="Q243" s="63" t="inlineStr">
+        <is>
+          <t>远征关卡01;办公室;开放办公;房间种类;30×40m;工位;文件柜;白板;图腾;绿植</t>
+        </is>
+      </c>
+      <c r="R243" s="90">
+        <f>LOWER(TRIM(C243)&amp;"|"&amp;TRIM(D243)&amp;"|"&amp;TRIM(E243)&amp;"|"&amp;TRIM(F243)&amp;"|"&amp;TRIM(H243)&amp;"|"&amp;TRIM(I243))</f>
+        <v/>
+      </c>
+      <c r="S243" s="90">
+        <f>IF(COUNTIF($R$6:$R$246,R243)&gt;1,"重复","唯一")</f>
+        <v/>
+      </c>
+      <c r="T243" s="90" t="inlineStr">
+        <is>
+          <t>4cf7138d0010405202d9cb9dd2aef0af9a676984ceeb90501b5a8d92304ed95f</t>
+        </is>
+      </c>
+      <c r="U243" s="63" t="inlineStr">
+        <is>
+          <t>摩斯拉</t>
+        </is>
+      </c>
+      <c r="V243" s="90" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="W243" s="63" t="inlineStr">
+        <is>
+          <t>用户设计（参考图 docs/v0.1/design/refs/expedition01/办公室01.jpg）</t>
+        </is>
+      </c>
+      <c r="X243" s="63" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Y243" s="63" t="inlineStr">
+        <is>
+          <t>服务远征关卡01 的 room_03（COMBAT，中心 -45/50）与 room_09（EVENT，中心 15/-45）；两房实测同为 office_60x70（30×40m）模板 ⇒ 共用一份房型源。白盒尺寸/门洞/墙高锁定，只做场景美术。未导 GLB、未接 Godot。</t>
+        </is>
+      </c>
+    </row>
+    <row r="244" ht="255" customHeight="1" s="60">
+      <c r="A244" s="90" t="inlineStr">
+        <is>
+          <t>ENV-EXPEDITION-L01-BRIDGE-ROOM</t>
+        </is>
+      </c>
+      <c r="B244" s="63" t="inlineStr">
+        <is>
+          <t>远征关卡01 通道桥 工字型 30×60m 房间种类源</t>
+        </is>
+      </c>
+      <c r="C244" s="63" t="inlineStr">
+        <is>
+          <t>场景</t>
+        </is>
+      </c>
+      <c r="D244" s="90" t="inlineStr">
+        <is>
+          <t>bridge_room</t>
+        </is>
+      </c>
+      <c r="E244" s="90" t="inlineStr">
+        <is>
+          <t>expedition_01_bridge_room</t>
+        </is>
+      </c>
+      <c r="F244" s="90" t="inlineStr">
+        <is>
+          <t>room_type</t>
+        </is>
+      </c>
+      <c r="G244" s="90" t="n"/>
+      <c r="H244" s="90" t="inlineStr">
+        <is>
+          <t>Top3D / Blender Z-up</t>
+        </is>
+      </c>
+      <c r="I244" s="90" t="inlineStr">
+        <is>
+          <t>scene_art / reference_derived</t>
+        </is>
+      </c>
+      <c r="J244" s="63" t="inlineStr">
+        <is>
+          <t>远征关卡01 专用；room_05 通道桥房间（工字型）</t>
+        </is>
+      </c>
+      <c r="K244" s="90" t="inlineStr">
+        <is>
+          <t>Blender源已完成</t>
+        </is>
+      </c>
+      <c r="L244" s="90" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="M244" s="90" t="inlineStr">
+        <is>
+          <t>v002</t>
+        </is>
+      </c>
+      <c r="N244" s="90" t="inlineStr">
+        <is>
+          <t>30×60×11.9m（工字型）；上层平台 30×60（Z∈[-0.32,0]）；中央跨桥 10×30m；下沉坑 30×30m、坑底 Z=-12.0；4 个下层服务标高；242 个独立组件包 / 314 输出网格 / 312370 面；门洞 2.2×2.5m；QA PASS（17 项断言）</t>
+        </is>
+      </c>
+      <c r="O244" s="90" t="inlineStr">
+        <is>
+          <t>assets/art/environments/tower_zones/expedition/source/room_types/bridge_room/v002/通道桥房间种类_工字型_30x60m_v002.blend</t>
+        </is>
+      </c>
+      <c r="P244" s="90" t="inlineStr">
+        <is>
+          <t>assets/art/environments/tower_zones/expedition/source/room_types/bridge_room/v002/build_bridge_room_v002.py；白盒 source/art/whitebox/tower_zones/expedition_01/v001/data/room_templates/bridge_60x50.json</t>
+        </is>
+      </c>
+      <c r="Q244" s="63" t="inlineStr">
+        <is>
+          <t>远征关卡01;通道桥;工字型;房间种类;30×60m;跨桥;下沉区;多层几何</t>
+        </is>
+      </c>
+      <c r="R244" s="90">
+        <f>LOWER(TRIM(C244)&amp;"|"&amp;TRIM(D244)&amp;"|"&amp;TRIM(E244)&amp;"|"&amp;TRIM(F244)&amp;"|"&amp;TRIM(H244)&amp;"|"&amp;TRIM(I244))</f>
+        <v/>
+      </c>
+      <c r="S244" s="90">
+        <f>IF(COUNTIF($R$6:$R$246,R244)&gt;1,"重复","唯一")</f>
+        <v/>
+      </c>
+      <c r="T244" s="90" t="inlineStr">
+        <is>
+          <t>7ba287e92a7a16fb7ee5234d027be6a969bdbccb4f12de5b741aaecfc7b2b59e</t>
+        </is>
+      </c>
+      <c r="U244" s="63" t="inlineStr">
+        <is>
+          <t>摩斯拉</t>
+        </is>
+      </c>
+      <c r="V244" s="90" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="W244" s="63" t="inlineStr">
+        <is>
+          <t>用户设计（参考图见 room_type_manifest.json 的 reference_image）</t>
+        </is>
+      </c>
+      <c r="X244" s="63" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Y244" s="63" t="inlineStr">
+        <is>
+          <t>服务远征关卡01 的 room_05（通道桥房间 30×60 · 工字型；转置姿态用 template_rotation_deg:90）。本批唯一需多层几何与碰撞的房型。v001 保留在同目录历史版本。未导 GLB、未接 Godot。</t>
+        </is>
+      </c>
+    </row>
+    <row r="245" ht="255" customHeight="1" s="60">
+      <c r="A245" s="90" t="inlineStr">
+        <is>
+          <t>ENV-EXPEDITION-L01-ROOM-STD-25X25</t>
+        </is>
+      </c>
+      <c r="B245" s="63" t="inlineStr">
+        <is>
+          <t>远征关卡01 标准房间 四墙平房 25×25m 房间种类源</t>
+        </is>
+      </c>
+      <c r="C245" s="63" t="inlineStr">
+        <is>
+          <t>场景</t>
+        </is>
+      </c>
+      <c r="D245" s="90" t="inlineStr">
+        <is>
+          <t>std_25x25</t>
+        </is>
+      </c>
+      <c r="E245" s="90" t="inlineStr">
+        <is>
+          <t>expedition_01_std_room</t>
+        </is>
+      </c>
+      <c r="F245" s="90" t="inlineStr">
+        <is>
+          <t>room_type</t>
+        </is>
+      </c>
+      <c r="G245" s="90" t="n"/>
+      <c r="H245" s="90" t="inlineStr">
+        <is>
+          <t>Top3D / Blender Z-up</t>
+        </is>
+      </c>
+      <c r="I245" s="90" t="inlineStr">
+        <is>
+          <t>scene_art / composed_from_linked_components</t>
+        </is>
+      </c>
+      <c r="J245" s="63" t="inlineStr">
+        <is>
+          <t>远征关卡01 专用；room_07 标准房间（25×25m）。本房型不自持几何：25 地砖 + 18 实墙 + 2 门墙 + 37 陈设共 82 个集合实例，全部 Library Link 自 office_room/v001 与 bridge_room/v002 两批已验收资产包</t>
+        </is>
+      </c>
+      <c r="K245" s="90" t="inlineStr">
+        <is>
+          <t>Blender源已完成</t>
+        </is>
+      </c>
+      <c r="L245" s="90" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="M245" s="90" t="inlineStr">
+        <is>
+          <t>v001</t>
+        </is>
+      </c>
+      <c r="N245" s="90" t="inlineStr">
+        <is>
+          <t>25×25×11.9m（5×5 个 5m 槽；四墙各 5 槽，墙槽心 ±10/±5/0）；82 个集合实例 / 引用 81 个已验收资产包 / 本文件自持网格 0；西·东墙 lane 0 对穿门洞 2.2×2.5m（净空底 0.30m、门楣 2.80m）；QA PASS（9 组断言）</t>
+        </is>
+      </c>
+      <c r="O245" s="90" t="inlineStr">
+        <is>
+          <t>assets/art/environments/tower_zones/expedition/source/room_types/std_25x25/v001/标准房间种类_四墙平房_25x25m_v001.blend</t>
+        </is>
+      </c>
+      <c r="P245" s="90" t="inlineStr">
+        <is>
+          <t>assets/art/environments/tower_zones/expedition/source/room_types/std_25x25/v001/build_std25_room_v001.py；摆位真源 同目录 std_25x25_v001.layout.json（由 _scratch/std25_layout/plan_std25_layout.py 算出）；白盒 source/art/whitebox/tower_zones/expedition_01/v001/data/room_templates/std_25x25.json</t>
+        </is>
+      </c>
+      <c r="Q245" s="63" t="inlineStr">
+        <is>
+          <t>远征关卡01;标准房间;四墙平房;房间种类;25×25m;组件拼装;LibraryLink;西东对穿;office_room;bridge_room</t>
+        </is>
+      </c>
+      <c r="R245" s="90">
+        <f>LOWER(TRIM(C245)&amp;"|"&amp;TRIM(D245)&amp;"|"&amp;TRIM(E245)&amp;"|"&amp;TRIM(F245)&amp;"|"&amp;TRIM(H245)&amp;"|"&amp;TRIM(I245))</f>
+        <v/>
+      </c>
+      <c r="S245" s="90">
+        <f>IF(COUNTIF($R$6:$R$246,R245)&gt;1,"重复","唯一")</f>
+        <v/>
+      </c>
+      <c r="T245" s="90" t="inlineStr">
+        <is>
+          <t>e5b69bef2804a6a46d44bef72b3b2e58f89bfe7440b4fa4a1551aa7ac7cf5974</t>
+        </is>
+      </c>
+      <c r="U245" s="63" t="inlineStr">
+        <is>
+          <t>摩斯拉</t>
+        </is>
+      </c>
+      <c r="V245" s="90" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="W245" s="63" t="inlineStr">
+        <is>
+          <t>用户设计（组件拼装；组件来源 office_room/v001 与 bridge_room/v002 两批已验收房型源）</t>
+        </is>
+      </c>
+      <c r="X245" s="63" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Y245" s="63" t="inlineStr">
+        <is>
+          <t>服务远征关卡01 的 room_07（标准房间，中心 −17.5/−87.5）。与 office/bridge 两行的语义差异：那两行是房型**自持几何**的组件源，本行是 skill 03 意义上的**实例布局源** ⇒ 自持几何 0、组件几何/材质/根原点一律不改、不缩放进位、不 Append 复制网格。与本房型摆位真源 std_25x25_v001.layout.json 配套的清单为同目录 component_inventory.json（记**被引用的**81 个外部资产包及本房用法）与 room_type_manifest.json。门位冻结为西/东墙 lane 0 对穿（依据设计页 §4.2.1 与参考图 08-标准房间.svg）。未导 GLB、未接 Godot。</t>
+        </is>
+      </c>
+    </row>
+    <row r="246" ht="255" customHeight="1" s="60">
+      <c r="A246" s="90" t="inlineStr">
+        <is>
+          <t>ENV-EXPEDITION-L01-ROOM-DB-70X50</t>
+        </is>
+      </c>
+      <c r="B246" s="63" t="inlineStr">
+        <is>
+          <t>远征关卡01 数据库房间 数据机房 40×30m 房间种类源</t>
+        </is>
+      </c>
+      <c r="C246" s="63" t="inlineStr">
+        <is>
+          <t>场景</t>
+        </is>
+      </c>
+      <c r="D246" s="90" t="inlineStr">
+        <is>
+          <t>db_room</t>
+        </is>
+      </c>
+      <c r="E246" s="90" t="inlineStr">
+        <is>
+          <t>expedition_01_db_room</t>
+        </is>
+      </c>
+      <c r="F246" s="90" t="inlineStr">
+        <is>
+          <t>room_type</t>
+        </is>
+      </c>
+      <c r="G246" s="90" t="n"/>
+      <c r="H246" s="90" t="inlineStr">
+        <is>
+          <t>Top3D / Blender Z-up</t>
+        </is>
+      </c>
+      <c r="I246" s="90" t="inlineStr">
+        <is>
+          <t>scene_art / reference_derived_with_linked_shell</t>
+        </is>
+      </c>
+      <c r="J246" s="63" t="inlineStr">
+        <is>
+          <t>远征关卡01 专用；room_02 / room_06 / room_10 三处实例共用同一房型源（同 db_70x50 模板）。本轮按参考图做 db_01 布局（主体 40×25 + 南侧中段外凸 10×5）；墙体与地砖 Library Link 复用 office_room/v001，其余 37 个组件包为数据库机房专属新制</t>
+        </is>
+      </c>
+      <c r="K246" s="90" t="inlineStr">
+        <is>
+          <t>Blender源已完成</t>
+        </is>
+      </c>
+      <c r="L246" s="90" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="M246" s="90" t="inlineStr">
+        <is>
+          <t>v001</t>
+        </is>
+      </c>
+      <c r="N246" s="90" t="inlineStr">
+        <is>
+          <t>40×30m 包围盒（8×6 个 5m 槽）；db_01 轮廓 = 主体 40×25 + 南侧中段外凸 10×5，占用 1050 m²（包围盒 1200 m²）；28 樘墙件 + 42 格地砖共 70 个集合实例，全部 Library Link 自 office_room/v001（本文件自持墙/砖网格 0）；37 个数据库机房专属组件包 / 49 输出网格 / 127164 面；门洞 2.2×2.5m（净空底 0.30m、门楣 2.80m）；16 个可开槽；QA PASS（26 项断言）</t>
+        </is>
+      </c>
+      <c r="O246" s="90" t="inlineStr">
+        <is>
+          <t>assets/art/environments/tower_zones/expedition/source/room_types/db_room/v001/数据库房间种类_数据机房_40x30m_v001.blend</t>
+        </is>
+      </c>
+      <c r="P246" s="90" t="inlineStr">
+        <is>
+          <t>assets/art/environments/tower_zones/expedition/source/room_types/db_room/v001/build_db_room_v001.py；白盒 source/art/whitebox/tower_zones/expedition_01/v001/data/room_templates/db_70x50.json；参考图 docs/v0.1/design/refs/expedition01/数据库房间01.jpg</t>
+        </is>
+      </c>
+      <c r="Q246" s="63" t="inlineStr">
+        <is>
+          <t>远征关卡01;数据库房间;数据机房;房间种类;40×30m;db_01;db_02;机柜;工作台;壁挂大屏;工具车;电缆盘;警示边带;LibraryLink;office_room</t>
+        </is>
+      </c>
+      <c r="R246" s="90">
+        <f>LOWER(TRIM(C246)&amp;"|"&amp;TRIM(D246)&amp;"|"&amp;TRIM(E246)&amp;"|"&amp;TRIM(F246)&amp;"|"&amp;TRIM(H246)&amp;"|"&amp;TRIM(I246))</f>
+        <v/>
+      </c>
+      <c r="S246" s="90">
+        <f>IF(COUNTIF($R$6:$R$246,R246)&gt;1,"重复","唯一")</f>
+        <v/>
+      </c>
+      <c r="T246" s="90" t="inlineStr">
+        <is>
+          <t>153eaa883b21b4489a3b5bb0b2d67a38419186ee0e7d1ff603bd3ad8f3c291a3</t>
+        </is>
+      </c>
+      <c r="U246" s="63" t="inlineStr">
+        <is>
+          <t>摩斯拉</t>
+        </is>
+      </c>
+      <c r="V246" s="90" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="W246" s="63" t="inlineStr">
+        <is>
+          <t>用户设计（参考图 docs/v0.1/design/refs/expedition01/数据库房间01.jpg；墙件与地砖复用 office_room/v001 已验收组件）</t>
+        </is>
+      </c>
+      <c r="X246" s="63" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Y246" s="63" t="inlineStr">
+        <is>
+          <t>服务远征关卡01 的 room_02 / room_06 / room_10（三处实例共用同一房型源）。本轮按参考图做 **db_01** 布局（主体 40×25 + 南侧中段外凸 10×5，面积 1050 m²）；同模板的另一内部布局 db_02（双缺角 15×10 / 15×5，面积 975 m²）按 room_type_manifest.json 显式标注为待另轮制作。与 office / bridge 两行的差别：墙件（28 樘）与地砖（42 格）**不重新制作**，改为 Library Link 引用 office_room/v001 的已验收组件包（本文件自持墙/砖网格 0、不 Append、不改组件几何/材质/根原点）；其余 37 个组件包（地面标识 / 格栅 / 设备坑抬升平台 / 西侧机柜列 7 台 / 中部机柜组 / 东墙 L 形工作台 / 西墙检修台 / 壁挂大屏组 / 红黄工具车 / 中央作业台 / 货箱堆场 / 重型货架 / 零件柜 / 电缆盘与线圈 / 花箱绿植 / 设备机架 / 墙面灯柱 / 顶部桥架管道风管灯具等）为数据库机房专属新制。未导 GLB、未接 Godot。</t>
         </is>
       </c>
     </row>
@@ -31294,17 +31778,14 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
-    <dataValidation sqref="C6:C242" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop" operator="between">
+    <dataValidation sqref="C6:C246" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"角色,敌人,武器,道具,场景,场景道具,基地资产包,UI,特效,音频"</formula1>
-      <formula2>0</formula2>
     </dataValidation>
-    <dataValidation sqref="K6:K242" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop" operator="between">
+    <dataValidation sqref="K6:K246" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"待制作,程序占位,已完成,原型已接入,弃用,旧资产已从正式基地移除,正式美术已接入,已优化并正式接入,Blender源已完成,已导入；优化完成,已从运行场景移除,白盒组件"</formula1>
-      <formula2>0</formula2>
     </dataValidation>
-    <dataValidation sqref="L6:L242" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop" operator="between">
+    <dataValidation sqref="L6:L246" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"P0,P1,P2,P3"</formula1>
-      <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
@@ -44766,7 +45247,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:G19"/>
+  <dimension ref="A1:G22"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.80859375" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="14" customWidth="1" style="59" min="1" max="1"/>
@@ -44793,6 +45274,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5" ht="15" customHeight="1" s="60">
       <c r="A5" s="66" t="inlineStr">
         <is>
@@ -45343,6 +45825,117 @@
         </is>
       </c>
       <c r="G19" s="119" t="inlineStr">
+        <is>
+          <t>摩斯拉</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" s="60">
+      <c r="A20" s="118" t="inlineStr">
+        <is>
+          <t>v0.1.14</t>
+        </is>
+      </c>
+      <c r="B20" s="118" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="C20" s="119" t="inlineStr">
+        <is>
+          <t>新增条目</t>
+        </is>
+      </c>
+      <c r="D20" s="119" t="inlineStr">
+        <is>
+          <t>关卡场景 / 远征关卡01</t>
+        </is>
+      </c>
+      <c r="E20" s="119" t="inlineStr">
+        <is>
+          <t>新增 ENV-EXPEDITION-L01-OFFICE-ROOM（远征关卡01 办公室 开放办公 30×40m 房间种类源，v001，服务 room_03 / room_09）与 ENV-EXPEDITION-L01-BRIDGE-ROOM（远征关卡01 通道桥 工字型 30×60m 房间种类源，v002，服务 room_05）。两者均由房型美术源制作完成（QA 分别 22 / 17 项断言全通过），白盒尺寸与门洞契约锁定，只做场景美术。</t>
+        </is>
+      </c>
+      <c r="F20" s="119" t="inlineStr">
+        <is>
+          <t>新增条目，不改动既有 AssetID / 路径 / 哈希；两行只落《资产主表》，《3D-场景通用》分页与专属摘要按「摘要锁死表须单独开事务」的规定留待导出 GLB / 接入 Godot 时一并处理。《总览》资产主表区间由 $…$242 扩到 $…$244，S 列查重结果逐行重算，DV 扩到第 244 行。</t>
+        </is>
+      </c>
+      <c r="G20" s="119" t="inlineStr">
+        <is>
+          <t>摩斯拉</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" s="60">
+      <c r="A21" s="118" t="inlineStr">
+        <is>
+          <t>v0.1.15</t>
+        </is>
+      </c>
+      <c r="B21" s="118" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="C21" s="119" t="inlineStr">
+        <is>
+          <t>新增条目</t>
+        </is>
+      </c>
+      <c r="D21" s="119" t="inlineStr">
+        <is>
+          <t>关卡场景 / 远征关卡01</t>
+        </is>
+      </c>
+      <c r="E21" s="119" t="inlineStr">
+        <is>
+          <t>新增 ENV-EXPEDITION-L01-ROOM-STD-25X25（远征关卡01 标准房间 四墙平房 25×25m 房间种类源，v001，服务 room_07）。本行是「实例布局源」而非「自持几何的组件源」：25 地砖 + 18 实墙 + 2 门墙 + 37 陈设共 82 个集合实例，全部 Library Link 自 office_room/v001（54 包）与 bridge_room/v002（27 包）两批已验收资产包，本文件自持网格 0、不 Append、不改组件几何/材质/根原点、无缩放。门位冻结为西/东墙 lane 0 对穿门洞（依据设计页 §4.2.1 与参考图 08-标准房间.svg）。结构契约校验 9 组断言全通过，渲染 6 机位验收。</t>
+        </is>
+      </c>
+      <c r="F21" s="119" t="inlineStr">
+        <is>
+          <t>新增条目，不改动既有 AssetID / 路径 / 哈希；本行只落《资产主表》，《3D-场景通用》分页（已声明「一行 = 一个实际存在的 Godot PackedScene」）按摘要锁死表规矩留待导出 GLB / 接入 Godot 时一并处理。《总览》资产主表区间由 $…$244 扩到 $…$245，S 列查重结果逐行重算，DV 扩到第 245 行；无损基线同步补录。</t>
+        </is>
+      </c>
+      <c r="G21" s="119" t="inlineStr">
+        <is>
+          <t>摩斯拉</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" s="60">
+      <c r="A22" s="118" t="inlineStr">
+        <is>
+          <t>v0.1.16</t>
+        </is>
+      </c>
+      <c r="B22" s="118" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="C22" s="119" t="inlineStr">
+        <is>
+          <t>新增条目</t>
+        </is>
+      </c>
+      <c r="D22" s="119" t="inlineStr">
+        <is>
+          <t>关卡场景 / 远征关卡01</t>
+        </is>
+      </c>
+      <c r="E22" s="119" t="inlineStr">
+        <is>
+          <t>新增 ENV-EXPEDITION-L01-ROOM-DB-70X50（远征关卡01 数据库房间 数据机房 40×30m 房间种类源，v001，服务 room_02 / room_06 / room_10）。本轮按参考图做 db_01 布局（主体 40×25 + 南侧中段外凸 10×5，占用 1050 m²）；**墙件 28 樘与地砖 42 格不自制**，改为 Library Link 引用 office_room/v001 的已验收组件包（本文件自持墙/砖网格 0）；其余 37 个组件包为数据库机房专属新制。结构契约校验 26 项断言全通过，渲染 6 机位验收。</t>
+        </is>
+      </c>
+      <c r="F22" s="119" t="inlineStr">
+        <is>
+          <t>新增条目，不改动既有 AssetID / 路径 / 哈希；本行只落《资产主表》，《3D-场景通用》分页（已声明「一行 = 一个实际存在的 Godot PackedScene」）按摘要锁死表规矩留待导出 GLB / 接入 Godot 时一并处理。《总览》资产主表区间由 $…$245 扩到 $…$246，S 列查重结果逐行重算，DV 扩到第 246 行；无损基线同步补录。</t>
+        </is>
+      </c>
+      <c r="G22" s="119" t="inlineStr">
         <is>
           <t>摩斯拉</t>
         </is>

</xml_diff>